<commit_message>
Ensure all cells have formulas in added rows
</commit_message>
<xml_diff>
--- a/te_algorithms/data/summary_table_drought.xlsx
+++ b/te_algorithms/data/summary_table_drought.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\azvoleff\Code\LandDegradation\trends.earth-algorithms\te_algorithms\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD081AF-6CE4-4E35-81A5-F47E6267993E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BAD0D3-4AEB-42C0-893D-8377A3F2D395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -418,7 +418,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -506,24 +506,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -546,13 +528,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -911,53 +893,53 @@
       </c>
     </row>
     <row r="3" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="44"/>
-      <c r="J3" s="44"/>
-      <c r="K3" s="44"/>
-      <c r="L3" s="44"/>
-      <c r="M3" s="44"/>
-      <c r="N3" s="44"/>
-      <c r="O3" s="44"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="38"/>
     </row>
     <row r="4" spans="1:15" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
     </row>
     <row r="5" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="D5" s="45" t="s">
+      <c r="D5" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="46"/>
-      <c r="F5" s="45" t="s">
+      <c r="E5" s="40"/>
+      <c r="F5" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="46"/>
-      <c r="H5" s="45" t="s">
+      <c r="G5" s="40"/>
+      <c r="H5" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="46"/>
-      <c r="J5" s="45" t="s">
+      <c r="I5" s="40"/>
+      <c r="J5" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="46"/>
-      <c r="L5" s="45" t="s">
+      <c r="K5" s="40"/>
+      <c r="L5" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="46"/>
-      <c r="N5" s="42" t="s">
+      <c r="M5" s="40"/>
+      <c r="N5" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="O5" s="43"/>
+      <c r="O5" s="37"/>
     </row>
     <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
@@ -1004,7 +986,7 @@
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="39"/>
+      <c r="A7" s="33"/>
       <c r="B7" s="12"/>
       <c r="C7" s="16" t="str">
         <f>IF(ISBLANK($B7),"",SUM(D7,F7,H7,J7,L7,N7))</f>
@@ -1042,7 +1024,7 @@
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="39"/>
+      <c r="A8" s="33"/>
       <c r="B8" s="12"/>
       <c r="C8" s="16" t="str">
         <f t="shared" ref="C8:C37" si="0">IF(ISBLANK($B8),"",SUM(D8,F8,H8,J8,L8,N8))</f>
@@ -1070,17 +1052,17 @@
       </c>
       <c r="L8" s="19"/>
       <c r="M8" s="7" t="str">
-        <f t="shared" ref="M8:O37" si="5">IF(ISBLANK($B8),"",L8/$C8)</f>
+        <f t="shared" ref="M8:M37" si="5">IF(ISBLANK($B8),"",L8/$C8)</f>
         <v/>
       </c>
       <c r="N8" s="26"/>
       <c r="O8" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="O8:O37" si="6">IF(ISBLANK($B8),"",N8/$C8)</f>
         <v/>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="39"/>
+      <c r="A9" s="33"/>
       <c r="B9" s="12"/>
       <c r="C9" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1113,12 +1095,12 @@
       </c>
       <c r="N9" s="26"/>
       <c r="O9" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="39"/>
+      <c r="A10" s="33"/>
       <c r="B10" s="12"/>
       <c r="C10" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1151,12 +1133,12 @@
       </c>
       <c r="N10" s="26"/>
       <c r="O10" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="39"/>
+      <c r="A11" s="33"/>
       <c r="B11" s="12"/>
       <c r="C11" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1189,12 +1171,12 @@
       </c>
       <c r="N11" s="26"/>
       <c r="O11" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="39"/>
+      <c r="A12" s="33"/>
       <c r="B12" s="12"/>
       <c r="C12" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1227,12 +1209,12 @@
       </c>
       <c r="N12" s="26"/>
       <c r="O12" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="39"/>
+      <c r="A13" s="33"/>
       <c r="B13" s="12"/>
       <c r="C13" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1265,12 +1247,12 @@
       </c>
       <c r="N13" s="26"/>
       <c r="O13" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="39"/>
+      <c r="A14" s="33"/>
       <c r="B14" s="12"/>
       <c r="C14" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1303,12 +1285,12 @@
       </c>
       <c r="N14" s="26"/>
       <c r="O14" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="39"/>
+      <c r="A15" s="33"/>
       <c r="B15" s="12"/>
       <c r="C15" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1341,12 +1323,12 @@
       </c>
       <c r="N15" s="26"/>
       <c r="O15" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="39"/>
+      <c r="A16" s="33"/>
       <c r="B16" s="12"/>
       <c r="C16" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1379,12 +1361,12 @@
       </c>
       <c r="N16" s="26"/>
       <c r="O16" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="39"/>
+      <c r="A17" s="33"/>
       <c r="B17" s="12"/>
       <c r="C17" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1417,12 +1399,12 @@
       </c>
       <c r="N17" s="26"/>
       <c r="O17" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="39"/>
+      <c r="A18" s="33"/>
       <c r="B18" s="12"/>
       <c r="C18" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1455,12 +1437,12 @@
       </c>
       <c r="N18" s="26"/>
       <c r="O18" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="39"/>
+      <c r="A19" s="33"/>
       <c r="B19" s="12"/>
       <c r="C19" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1493,12 +1475,12 @@
       </c>
       <c r="N19" s="26"/>
       <c r="O19" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="39"/>
+      <c r="A20" s="33"/>
       <c r="B20" s="12"/>
       <c r="C20" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1531,12 +1513,12 @@
       </c>
       <c r="N20" s="26"/>
       <c r="O20" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="39"/>
+      <c r="A21" s="33"/>
       <c r="B21" s="12"/>
       <c r="C21" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1569,12 +1551,12 @@
       </c>
       <c r="N21" s="26"/>
       <c r="O21" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="39"/>
+      <c r="A22" s="33"/>
       <c r="B22" s="12"/>
       <c r="C22" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1607,12 +1589,12 @@
       </c>
       <c r="N22" s="26"/>
       <c r="O22" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="39"/>
+      <c r="A23" s="33"/>
       <c r="B23" s="12"/>
       <c r="C23" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1645,12 +1627,12 @@
       </c>
       <c r="N23" s="26"/>
       <c r="O23" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="39"/>
+      <c r="A24" s="33"/>
       <c r="B24" s="12"/>
       <c r="C24" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1683,12 +1665,12 @@
       </c>
       <c r="N24" s="26"/>
       <c r="O24" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="39"/>
+      <c r="A25" s="33"/>
       <c r="B25" s="12"/>
       <c r="C25" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1721,148 +1703,316 @@
       </c>
       <c r="N25" s="26"/>
       <c r="O25" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="33"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D26" s="19"/>
+      <c r="E26" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="F26" s="19"/>
+      <c r="G26" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H26" s="22"/>
+      <c r="I26" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="J26" s="19"/>
+      <c r="K26" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="L26" s="19"/>
+      <c r="M26" s="7" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="39"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="22"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="19"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="19"/>
-      <c r="M26" s="7"/>
       <c r="N26" s="26"/>
-      <c r="O26" s="27"/>
+      <c r="O26" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="39"/>
+      <c r="A27" s="33"/>
       <c r="B27" s="12"/>
-      <c r="C27" s="16"/>
+      <c r="C27" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D27" s="19"/>
-      <c r="E27" s="7"/>
+      <c r="E27" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F27" s="19"/>
-      <c r="G27" s="7"/>
+      <c r="G27" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H27" s="22"/>
-      <c r="I27" s="7"/>
+      <c r="I27" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J27" s="19"/>
-      <c r="K27" s="7"/>
+      <c r="K27" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L27" s="19"/>
-      <c r="M27" s="7"/>
+      <c r="M27" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N27" s="26"/>
-      <c r="O27" s="27"/>
+      <c r="O27" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="39"/>
+      <c r="A28" s="33"/>
       <c r="B28" s="12"/>
-      <c r="C28" s="16"/>
+      <c r="C28" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D28" s="19"/>
-      <c r="E28" s="7"/>
+      <c r="E28" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F28" s="19"/>
-      <c r="G28" s="7"/>
+      <c r="G28" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H28" s="22"/>
-      <c r="I28" s="7"/>
+      <c r="I28" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J28" s="19"/>
-      <c r="K28" s="7"/>
+      <c r="K28" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L28" s="19"/>
-      <c r="M28" s="7"/>
+      <c r="M28" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N28" s="26"/>
-      <c r="O28" s="27"/>
+      <c r="O28" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="39"/>
+      <c r="A29" s="33"/>
       <c r="B29" s="12"/>
-      <c r="C29" s="16"/>
+      <c r="C29" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D29" s="19"/>
-      <c r="E29" s="7"/>
+      <c r="E29" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F29" s="19"/>
-      <c r="G29" s="7"/>
+      <c r="G29" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H29" s="22"/>
-      <c r="I29" s="7"/>
+      <c r="I29" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J29" s="19"/>
-      <c r="K29" s="7"/>
+      <c r="K29" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L29" s="19"/>
-      <c r="M29" s="7"/>
+      <c r="M29" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N29" s="26"/>
-      <c r="O29" s="27"/>
+      <c r="O29" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="39"/>
+      <c r="A30" s="33"/>
       <c r="B30" s="12"/>
-      <c r="C30" s="16"/>
+      <c r="C30" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D30" s="19"/>
-      <c r="E30" s="7"/>
+      <c r="E30" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F30" s="19"/>
-      <c r="G30" s="7"/>
+      <c r="G30" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H30" s="22"/>
-      <c r="I30" s="7"/>
+      <c r="I30" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J30" s="19"/>
-      <c r="K30" s="7"/>
+      <c r="K30" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L30" s="19"/>
-      <c r="M30" s="7"/>
+      <c r="M30" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N30" s="26"/>
-      <c r="O30" s="27"/>
+      <c r="O30" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="39"/>
+      <c r="A31" s="33"/>
       <c r="B31" s="12"/>
-      <c r="C31" s="16"/>
+      <c r="C31" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D31" s="19"/>
-      <c r="E31" s="7"/>
+      <c r="E31" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F31" s="19"/>
-      <c r="G31" s="7"/>
+      <c r="G31" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H31" s="22"/>
-      <c r="I31" s="7"/>
+      <c r="I31" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J31" s="19"/>
-      <c r="K31" s="7"/>
+      <c r="K31" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L31" s="19"/>
-      <c r="M31" s="7"/>
+      <c r="M31" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N31" s="26"/>
-      <c r="O31" s="27"/>
+      <c r="O31" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="39"/>
+      <c r="A32" s="33"/>
       <c r="B32" s="12"/>
-      <c r="C32" s="16"/>
+      <c r="C32" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D32" s="19"/>
-      <c r="E32" s="7"/>
+      <c r="E32" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F32" s="19"/>
-      <c r="G32" s="7"/>
+      <c r="G32" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H32" s="22"/>
-      <c r="I32" s="7"/>
+      <c r="I32" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J32" s="19"/>
-      <c r="K32" s="7"/>
+      <c r="K32" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L32" s="19"/>
-      <c r="M32" s="7"/>
+      <c r="M32" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N32" s="26"/>
-      <c r="O32" s="27"/>
+      <c r="O32" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="39"/>
+      <c r="A33" s="33"/>
       <c r="B33" s="12"/>
-      <c r="C33" s="16"/>
+      <c r="C33" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D33" s="19"/>
-      <c r="E33" s="7"/>
+      <c r="E33" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F33" s="19"/>
-      <c r="G33" s="7"/>
+      <c r="G33" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H33" s="22"/>
-      <c r="I33" s="7"/>
+      <c r="I33" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J33" s="19"/>
-      <c r="K33" s="7"/>
+      <c r="K33" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L33" s="19"/>
-      <c r="M33" s="7"/>
+      <c r="M33" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N33" s="26"/>
-      <c r="O33" s="27"/>
+      <c r="O33" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34" s="39"/>
+      <c r="A34" s="33"/>
       <c r="B34" s="12"/>
       <c r="C34" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1895,12 +2045,12 @@
       </c>
       <c r="N34" s="26"/>
       <c r="O34" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="39"/>
+      <c r="A35" s="33"/>
       <c r="B35" s="12"/>
       <c r="C35" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1933,12 +2083,12 @@
       </c>
       <c r="N35" s="26"/>
       <c r="O35" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36" s="39"/>
+      <c r="A36" s="33"/>
       <c r="B36" s="12"/>
       <c r="C36" s="16" t="str">
         <f t="shared" si="0"/>
@@ -1971,12 +2121,12 @@
       </c>
       <c r="N36" s="26"/>
       <c r="O36" s="27" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="37" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="39"/>
+      <c r="A37" s="33"/>
       <c r="B37" s="12"/>
       <c r="C37" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2009,7 +2159,7 @@
       </c>
       <c r="N37" s="28"/>
       <c r="O37" s="29" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
@@ -2024,38 +2174,38 @@
       <c r="H38" s="21"/>
     </row>
     <row r="39" spans="1:15" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="40" t="s">
+      <c r="A39" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B39" s="40"/>
-      <c r="C39" s="40"/>
-      <c r="D39" s="40"/>
-      <c r="E39" s="40"/>
-      <c r="F39" s="40"/>
-      <c r="G39" s="40"/>
-      <c r="H39" s="40"/>
-      <c r="I39" s="40"/>
-      <c r="J39" s="40"/>
-      <c r="K39" s="40"/>
-      <c r="L39" s="40"/>
-      <c r="M39" s="40"/>
+      <c r="B39" s="34"/>
+      <c r="C39" s="34"/>
+      <c r="D39" s="34"/>
+      <c r="E39" s="34"/>
+      <c r="F39" s="34"/>
+      <c r="G39" s="34"/>
+      <c r="H39" s="34"/>
+      <c r="I39" s="34"/>
+      <c r="J39" s="34"/>
+      <c r="K39" s="34"/>
+      <c r="L39" s="34"/>
+      <c r="M39" s="34"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="41" t="s">
+      <c r="A41" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B41" s="41"/>
-      <c r="C41" s="41"/>
-      <c r="D41" s="41"/>
-      <c r="E41" s="41"/>
-      <c r="F41" s="41"/>
-      <c r="G41" s="41"/>
-      <c r="H41" s="41"/>
-      <c r="I41" s="41"/>
-      <c r="J41" s="41"/>
-      <c r="K41" s="41"/>
-      <c r="L41" s="41"/>
-      <c r="M41" s="41"/>
+      <c r="B41" s="35"/>
+      <c r="C41" s="35"/>
+      <c r="D41" s="35"/>
+      <c r="E41" s="35"/>
+      <c r="F41" s="35"/>
+      <c r="G41" s="35"/>
+      <c r="H41" s="35"/>
+      <c r="I41" s="35"/>
+      <c r="J41" s="35"/>
+      <c r="K41" s="35"/>
+      <c r="L41" s="35"/>
+      <c r="M41" s="35"/>
       <c r="N41"/>
       <c r="O41"/>
     </row>
@@ -2079,7 +2229,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:O115"/>
+  <dimension ref="A1:O113"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" customWidth="1"/>
@@ -2110,53 +2260,53 @@
       </c>
     </row>
     <row r="3" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
-      <c r="L3" s="47"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="47"/>
-      <c r="O3" s="47"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="42"/>
+      <c r="N3" s="42"/>
+      <c r="O3" s="42"/>
     </row>
     <row r="4" spans="1:15" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
     </row>
     <row r="5" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="D5" s="45" t="s">
+      <c r="D5" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="46"/>
-      <c r="F5" s="45" t="s">
+      <c r="E5" s="40"/>
+      <c r="F5" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="46"/>
-      <c r="H5" s="45" t="s">
+      <c r="G5" s="40"/>
+      <c r="H5" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="46"/>
-      <c r="J5" s="45" t="s">
+      <c r="I5" s="40"/>
+      <c r="J5" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="46"/>
-      <c r="L5" s="45" t="s">
+      <c r="K5" s="40"/>
+      <c r="L5" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="46"/>
-      <c r="N5" s="42" t="s">
+      <c r="M5" s="40"/>
+      <c r="N5" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="O5" s="43"/>
+      <c r="O5" s="37"/>
     </row>
     <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
@@ -2203,7 +2353,7 @@
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="39"/>
+      <c r="A7" s="33"/>
       <c r="B7" s="12"/>
       <c r="C7" s="16" t="str">
         <f>IF(ISBLANK($B7),"",SUM(D7,F7,H7,J7,L7,N7))</f>
@@ -2241,7 +2391,7 @@
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="39"/>
+      <c r="A8" s="33"/>
       <c r="B8" s="12"/>
       <c r="C8" s="16" t="str">
         <f t="shared" ref="C8:C37" si="0">IF(ISBLANK($B8),"",SUM(D8,F8,H8,J8,L8,N8))</f>
@@ -2279,7 +2429,7 @@
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="39"/>
+      <c r="A9" s="33"/>
       <c r="B9" s="12"/>
       <c r="C9" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2317,7 +2467,7 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="39"/>
+      <c r="A10" s="33"/>
       <c r="B10" s="12"/>
       <c r="C10" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2355,7 +2505,7 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="39"/>
+      <c r="A11" s="33"/>
       <c r="B11" s="12"/>
       <c r="C11" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2393,7 +2543,7 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="39"/>
+      <c r="A12" s="33"/>
       <c r="B12" s="12"/>
       <c r="C12" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2431,7 +2581,7 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="39"/>
+      <c r="A13" s="33"/>
       <c r="B13" s="12"/>
       <c r="C13" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2469,7 +2619,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="39"/>
+      <c r="A14" s="33"/>
       <c r="B14" s="12"/>
       <c r="C14" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2507,7 +2657,7 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="39"/>
+      <c r="A15" s="33"/>
       <c r="B15" s="12"/>
       <c r="C15" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2545,7 +2695,7 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="39"/>
+      <c r="A16" s="33"/>
       <c r="B16" s="12"/>
       <c r="C16" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2583,7 +2733,7 @@
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="39"/>
+      <c r="A17" s="33"/>
       <c r="B17" s="12"/>
       <c r="C17" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2621,7 +2771,7 @@
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="39"/>
+      <c r="A18" s="33"/>
       <c r="B18" s="12"/>
       <c r="C18" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2659,7 +2809,7 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="39"/>
+      <c r="A19" s="33"/>
       <c r="B19" s="12"/>
       <c r="C19" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2697,7 +2847,7 @@
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="39"/>
+      <c r="A20" s="33"/>
       <c r="B20" s="12"/>
       <c r="C20" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2735,7 +2885,7 @@
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="39"/>
+      <c r="A21" s="33"/>
       <c r="B21" s="12"/>
       <c r="C21" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2773,7 +2923,7 @@
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="39"/>
+      <c r="A22" s="33"/>
       <c r="B22" s="12"/>
       <c r="C22" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2811,126 +2961,273 @@
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="39"/>
+      <c r="A23" s="33"/>
       <c r="B23" s="12"/>
-      <c r="C23" s="16"/>
+      <c r="C23" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D23" s="19"/>
-      <c r="E23" s="7"/>
+      <c r="E23" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F23" s="19"/>
-      <c r="G23" s="7"/>
+      <c r="G23" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H23" s="22"/>
-      <c r="I23" s="7"/>
+      <c r="I23" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J23" s="19"/>
-      <c r="K23" s="7"/>
+      <c r="K23" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L23" s="19"/>
-      <c r="M23" s="7"/>
+      <c r="M23" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N23" s="26"/>
-      <c r="O23" s="27"/>
+      <c r="O23" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="39"/>
+      <c r="A24" s="33"/>
       <c r="B24" s="12"/>
-      <c r="C24" s="16"/>
+      <c r="C24" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D24" s="19"/>
-      <c r="E24" s="7"/>
+      <c r="E24" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F24" s="19"/>
-      <c r="G24" s="7"/>
+      <c r="G24" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H24" s="22"/>
-      <c r="I24" s="7"/>
+      <c r="I24" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J24" s="19"/>
-      <c r="K24" s="7"/>
+      <c r="K24" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L24" s="19"/>
-      <c r="M24" s="7"/>
+      <c r="M24" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N24" s="26"/>
-      <c r="O24" s="27"/>
+      <c r="O24" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="39"/>
+      <c r="A25" s="33"/>
       <c r="B25" s="12"/>
-      <c r="C25" s="16"/>
+      <c r="C25" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D25" s="19"/>
-      <c r="E25" s="7"/>
+      <c r="E25" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F25" s="19"/>
-      <c r="G25" s="7"/>
+      <c r="G25" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H25" s="22"/>
-      <c r="I25" s="7"/>
+      <c r="I25" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J25" s="19"/>
-      <c r="K25" s="7"/>
+      <c r="K25" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L25" s="19"/>
-      <c r="M25" s="7"/>
+      <c r="M25" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N25" s="26"/>
-      <c r="O25" s="27"/>
+      <c r="O25" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="39"/>
+      <c r="A26" s="33"/>
       <c r="B26" s="12"/>
-      <c r="C26" s="16"/>
+      <c r="C26" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D26" s="19"/>
-      <c r="E26" s="7"/>
+      <c r="E26" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F26" s="19"/>
-      <c r="G26" s="7"/>
+      <c r="G26" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H26" s="22"/>
-      <c r="I26" s="7"/>
+      <c r="I26" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J26" s="19"/>
-      <c r="K26" s="7"/>
+      <c r="K26" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L26" s="19"/>
-      <c r="M26" s="7"/>
+      <c r="M26" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N26" s="26"/>
-      <c r="O26" s="27"/>
+      <c r="O26" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="39"/>
+      <c r="A27" s="33"/>
       <c r="B27" s="12"/>
-      <c r="C27" s="16"/>
+      <c r="C27" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D27" s="19"/>
-      <c r="E27" s="7"/>
+      <c r="E27" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F27" s="19"/>
-      <c r="G27" s="7"/>
+      <c r="G27" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H27" s="22"/>
-      <c r="I27" s="7"/>
+      <c r="I27" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J27" s="19"/>
-      <c r="K27" s="7"/>
+      <c r="K27" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L27" s="19"/>
-      <c r="M27" s="7"/>
+      <c r="M27" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N27" s="26"/>
-      <c r="O27" s="27"/>
+      <c r="O27" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="39"/>
+      <c r="A28" s="33"/>
       <c r="B28" s="12"/>
-      <c r="C28" s="16"/>
+      <c r="C28" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D28" s="19"/>
-      <c r="E28" s="7"/>
+      <c r="E28" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F28" s="19"/>
-      <c r="G28" s="7"/>
+      <c r="G28" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H28" s="22"/>
-      <c r="I28" s="7"/>
+      <c r="I28" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J28" s="19"/>
-      <c r="K28" s="7"/>
+      <c r="K28" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L28" s="19"/>
-      <c r="M28" s="7"/>
+      <c r="M28" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N28" s="26"/>
-      <c r="O28" s="27"/>
+      <c r="O28" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="39"/>
+      <c r="A29" s="33"/>
       <c r="B29" s="12"/>
-      <c r="C29" s="16"/>
+      <c r="C29" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D29" s="19"/>
-      <c r="E29" s="7"/>
+      <c r="E29" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F29" s="19"/>
-      <c r="G29" s="7"/>
+      <c r="G29" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H29" s="22"/>
-      <c r="I29" s="7"/>
+      <c r="I29" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J29" s="19"/>
-      <c r="K29" s="7"/>
+      <c r="K29" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L29" s="19"/>
-      <c r="M29" s="7"/>
+      <c r="M29" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N29" s="26"/>
-      <c r="O29" s="27"/>
+      <c r="O29" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="39"/>
+      <c r="A30" s="33"/>
       <c r="B30" s="12"/>
       <c r="C30" s="16" t="str">
         <f t="shared" si="0"/>
@@ -2968,7 +3265,7 @@
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="39"/>
+      <c r="A31" s="33"/>
       <c r="B31" s="12"/>
       <c r="C31" s="16" t="str">
         <f t="shared" si="0"/>
@@ -3006,24 +3303,45 @@
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="39"/>
+      <c r="A32" s="33"/>
       <c r="B32" s="12"/>
-      <c r="C32" s="16"/>
+      <c r="C32" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="D32" s="19"/>
-      <c r="E32" s="7"/>
+      <c r="E32" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="F32" s="19"/>
-      <c r="G32" s="7"/>
+      <c r="G32" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="H32" s="22"/>
-      <c r="I32" s="7"/>
+      <c r="I32" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J32" s="19"/>
-      <c r="K32" s="7"/>
+      <c r="K32" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
       <c r="L32" s="19"/>
-      <c r="M32" s="7"/>
+      <c r="M32" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
       <c r="N32" s="26"/>
-      <c r="O32" s="27"/>
+      <c r="O32" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="39"/>
+      <c r="A33" s="33"/>
       <c r="B33" s="12"/>
       <c r="C33" s="16" t="str">
         <f t="shared" si="0"/>
@@ -3061,7 +3379,7 @@
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34" s="39"/>
+      <c r="A34" s="33"/>
       <c r="B34" s="12"/>
       <c r="C34" s="16" t="str">
         <f t="shared" si="0"/>
@@ -3099,7 +3417,7 @@
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="39"/>
+      <c r="A35" s="33"/>
       <c r="B35" s="12"/>
       <c r="C35" s="16" t="str">
         <f t="shared" si="0"/>
@@ -3137,7 +3455,7 @@
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36" s="39"/>
+      <c r="A36" s="33"/>
       <c r="B36" s="12"/>
       <c r="C36" s="16" t="str">
         <f t="shared" si="0"/>
@@ -3175,7 +3493,7 @@
       </c>
     </row>
     <row r="37" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="39"/>
+      <c r="A37" s="33"/>
       <c r="B37" s="12"/>
       <c r="C37" s="16" t="str">
         <f t="shared" si="0"/>
@@ -3229,23 +3547,23 @@
       <c r="O38"/>
     </row>
     <row r="39" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A39" s="48" t="s">
+      <c r="A39" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="B39" s="48"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="48"/>
-      <c r="E39" s="48"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="48"/>
-      <c r="H39" s="48"/>
-      <c r="I39" s="48"/>
-      <c r="J39" s="48"/>
-      <c r="K39" s="48"/>
-      <c r="L39" s="48"/>
-      <c r="M39" s="48"/>
-      <c r="N39" s="48"/>
-      <c r="O39" s="48"/>
+      <c r="B39" s="43"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="43"/>
+      <c r="I39" s="43"/>
+      <c r="J39" s="43"/>
+      <c r="K39" s="43"/>
+      <c r="L39" s="43"/>
+      <c r="M39" s="43"/>
+      <c r="N39" s="43"/>
+      <c r="O39" s="43"/>
     </row>
     <row r="40" spans="1:15" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
@@ -3254,30 +3572,30 @@
       <c r="A41" s="1"/>
       <c r="B41" s="10"/>
       <c r="C41" s="14"/>
-      <c r="D41" s="45" t="s">
+      <c r="D41" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="E41" s="46"/>
-      <c r="F41" s="45" t="s">
+      <c r="E41" s="40"/>
+      <c r="F41" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="G41" s="46"/>
-      <c r="H41" s="45" t="s">
+      <c r="G41" s="40"/>
+      <c r="H41" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="I41" s="46"/>
-      <c r="J41" s="45" t="s">
+      <c r="I41" s="40"/>
+      <c r="J41" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="K41" s="46"/>
-      <c r="L41" s="45" t="s">
+      <c r="K41" s="40"/>
+      <c r="L41" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="M41" s="46"/>
-      <c r="N41" s="42" t="s">
+      <c r="M41" s="40"/>
+      <c r="N41" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="O41" s="43"/>
+      <c r="O41" s="37"/>
     </row>
     <row r="42" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B42" s="11" t="s">
@@ -3324,7 +3642,7 @@
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="39"/>
+      <c r="A43" s="33"/>
       <c r="B43" s="12"/>
       <c r="C43" s="16" t="str">
         <f>IF(ISBLANK($B43),"",SUM(D43,F43,H43,J43,L43,N43))</f>
@@ -3362,7 +3680,7 @@
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44" s="39"/>
+      <c r="A44" s="33"/>
       <c r="B44" s="12"/>
       <c r="C44" s="16" t="str">
         <f t="shared" ref="C44:C73" si="7">IF(ISBLANK($B44),"",SUM(D44,F44,H44,J44,L44,N44))</f>
@@ -3400,7 +3718,7 @@
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45" s="39"/>
+      <c r="A45" s="33"/>
       <c r="B45" s="12"/>
       <c r="C45" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3438,7 +3756,7 @@
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A46" s="39"/>
+      <c r="A46" s="33"/>
       <c r="B46" s="12"/>
       <c r="C46" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3476,7 +3794,7 @@
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A47" s="39"/>
+      <c r="A47" s="33"/>
       <c r="B47" s="12"/>
       <c r="C47" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3514,7 +3832,7 @@
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="39"/>
+      <c r="A48" s="33"/>
       <c r="B48" s="12"/>
       <c r="C48" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3552,7 +3870,7 @@
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A49" s="39"/>
+      <c r="A49" s="33"/>
       <c r="B49" s="12"/>
       <c r="C49" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3590,7 +3908,7 @@
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A50" s="39"/>
+      <c r="A50" s="33"/>
       <c r="B50" s="12"/>
       <c r="C50" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3628,7 +3946,7 @@
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A51" s="39"/>
+      <c r="A51" s="33"/>
       <c r="B51" s="12"/>
       <c r="C51" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3666,7 +3984,7 @@
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A52" s="39"/>
+      <c r="A52" s="33"/>
       <c r="B52" s="12"/>
       <c r="C52" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3704,7 +4022,7 @@
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A53" s="39"/>
+      <c r="A53" s="33"/>
       <c r="B53" s="12"/>
       <c r="C53" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3742,7 +4060,7 @@
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A54" s="39"/>
+      <c r="A54" s="33"/>
       <c r="B54" s="12"/>
       <c r="C54" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3780,7 +4098,7 @@
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A55" s="39"/>
+      <c r="A55" s="33"/>
       <c r="B55" s="12"/>
       <c r="C55" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3818,7 +4136,7 @@
       </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A56" s="39"/>
+      <c r="A56" s="33"/>
       <c r="B56" s="12"/>
       <c r="C56" s="16" t="str">
         <f t="shared" si="7"/>
@@ -3856,143 +4174,311 @@
       </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A57" s="39"/>
+      <c r="A57" s="33"/>
       <c r="B57" s="12"/>
-      <c r="C57" s="16"/>
+      <c r="C57" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="D57" s="19"/>
-      <c r="E57" s="7"/>
+      <c r="E57" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="F57" s="19"/>
-      <c r="G57" s="7"/>
+      <c r="G57" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
       <c r="H57" s="22"/>
-      <c r="I57" s="7"/>
+      <c r="I57" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
       <c r="J57" s="19"/>
-      <c r="K57" s="7"/>
+      <c r="K57" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
       <c r="L57" s="19"/>
-      <c r="M57" s="7"/>
+      <c r="M57" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
       <c r="N57" s="26"/>
-      <c r="O57" s="27"/>
+      <c r="O57" s="27" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A58" s="39"/>
+      <c r="A58" s="33"/>
       <c r="B58" s="12"/>
-      <c r="C58" s="16"/>
+      <c r="C58" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="D58" s="19"/>
-      <c r="E58" s="7"/>
+      <c r="E58" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="F58" s="19"/>
-      <c r="G58" s="7"/>
+      <c r="G58" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
       <c r="H58" s="22"/>
-      <c r="I58" s="7"/>
+      <c r="I58" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
       <c r="J58" s="19"/>
-      <c r="K58" s="7"/>
+      <c r="K58" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
       <c r="L58" s="19"/>
-      <c r="M58" s="7"/>
+      <c r="M58" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
       <c r="N58" s="26"/>
-      <c r="O58" s="27"/>
+      <c r="O58" s="27" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A59" s="39"/>
+      <c r="A59" s="33"/>
       <c r="B59" s="12"/>
-      <c r="C59" s="16"/>
+      <c r="C59" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="D59" s="19"/>
-      <c r="E59" s="7"/>
+      <c r="E59" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="F59" s="19"/>
-      <c r="G59" s="7"/>
+      <c r="G59" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
       <c r="H59" s="22"/>
-      <c r="I59" s="7"/>
+      <c r="I59" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
       <c r="J59" s="19"/>
-      <c r="K59" s="7"/>
+      <c r="K59" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
       <c r="L59" s="19"/>
-      <c r="M59" s="7"/>
+      <c r="M59" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
       <c r="N59" s="26"/>
-      <c r="O59" s="27"/>
+      <c r="O59" s="27" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A60" s="39"/>
+      <c r="A60" s="33"/>
       <c r="B60" s="12"/>
-      <c r="C60" s="16"/>
+      <c r="C60" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="D60" s="19"/>
-      <c r="E60" s="7"/>
+      <c r="E60" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="F60" s="19"/>
-      <c r="G60" s="7"/>
+      <c r="G60" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
       <c r="H60" s="22"/>
-      <c r="I60" s="7"/>
+      <c r="I60" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
       <c r="J60" s="19"/>
-      <c r="K60" s="7"/>
+      <c r="K60" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
       <c r="L60" s="19"/>
-      <c r="M60" s="7"/>
+      <c r="M60" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
       <c r="N60" s="26"/>
-      <c r="O60" s="27"/>
+      <c r="O60" s="27" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A61" s="39"/>
+      <c r="A61" s="33"/>
       <c r="B61" s="12"/>
-      <c r="C61" s="16"/>
+      <c r="C61" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="D61" s="19"/>
-      <c r="E61" s="7"/>
+      <c r="E61" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="F61" s="19"/>
-      <c r="G61" s="7"/>
+      <c r="G61" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
       <c r="H61" s="22"/>
-      <c r="I61" s="7"/>
+      <c r="I61" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
       <c r="J61" s="19"/>
-      <c r="K61" s="7"/>
+      <c r="K61" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
       <c r="L61" s="19"/>
-      <c r="M61" s="7"/>
+      <c r="M61" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
       <c r="N61" s="26"/>
-      <c r="O61" s="27"/>
+      <c r="O61" s="27" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A62" s="39"/>
+      <c r="A62" s="33"/>
       <c r="B62" s="12"/>
-      <c r="C62" s="16"/>
+      <c r="C62" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="D62" s="19"/>
-      <c r="E62" s="7"/>
+      <c r="E62" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="F62" s="19"/>
-      <c r="G62" s="7"/>
+      <c r="G62" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
       <c r="H62" s="22"/>
-      <c r="I62" s="7"/>
+      <c r="I62" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
       <c r="J62" s="19"/>
-      <c r="K62" s="7"/>
+      <c r="K62" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
       <c r="L62" s="19"/>
-      <c r="M62" s="7"/>
+      <c r="M62" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
       <c r="N62" s="26"/>
-      <c r="O62" s="27"/>
+      <c r="O62" s="27" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A63" s="39"/>
+      <c r="A63" s="33"/>
       <c r="B63" s="12"/>
-      <c r="C63" s="16"/>
+      <c r="C63" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="D63" s="19"/>
-      <c r="E63" s="7"/>
+      <c r="E63" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="F63" s="19"/>
-      <c r="G63" s="7"/>
+      <c r="G63" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
       <c r="H63" s="22"/>
-      <c r="I63" s="7"/>
+      <c r="I63" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
       <c r="J63" s="19"/>
-      <c r="K63" s="7"/>
+      <c r="K63" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
       <c r="L63" s="19"/>
-      <c r="M63" s="7"/>
+      <c r="M63" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
       <c r="N63" s="26"/>
-      <c r="O63" s="27"/>
+      <c r="O63" s="27" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A64" s="39"/>
+      <c r="A64" s="33"/>
       <c r="B64" s="12"/>
-      <c r="C64" s="16"/>
+      <c r="C64" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="D64" s="19"/>
-      <c r="E64" s="7"/>
+      <c r="E64" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="F64" s="19"/>
-      <c r="G64" s="7"/>
+      <c r="G64" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
       <c r="H64" s="22"/>
-      <c r="I64" s="7"/>
+      <c r="I64" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
       <c r="J64" s="19"/>
-      <c r="K64" s="7"/>
+      <c r="K64" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
       <c r="L64" s="19"/>
-      <c r="M64" s="7"/>
+      <c r="M64" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
       <c r="N64" s="26"/>
-      <c r="O64" s="27"/>
+      <c r="O64" s="27" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A65" s="39"/>
+      <c r="A65" s="33"/>
       <c r="B65" s="12"/>
       <c r="C65" s="16" t="str">
         <f t="shared" si="7"/>
@@ -4030,7 +4516,7 @@
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A66" s="39"/>
+      <c r="A66" s="33"/>
       <c r="B66" s="12"/>
       <c r="C66" s="16" t="str">
         <f t="shared" si="7"/>
@@ -4068,7 +4554,7 @@
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A67" s="39"/>
+      <c r="A67" s="33"/>
       <c r="B67" s="12"/>
       <c r="C67" s="16" t="str">
         <f t="shared" si="7"/>
@@ -4106,7 +4592,7 @@
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A68" s="39"/>
+      <c r="A68" s="33"/>
       <c r="B68" s="12"/>
       <c r="C68" s="16" t="str">
         <f t="shared" si="7"/>
@@ -4144,7 +4630,7 @@
       </c>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A69" s="39"/>
+      <c r="A69" s="33"/>
       <c r="B69" s="12"/>
       <c r="C69" s="16" t="str">
         <f t="shared" si="7"/>
@@ -4182,7 +4668,7 @@
       </c>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A70" s="39"/>
+      <c r="A70" s="33"/>
       <c r="B70" s="12"/>
       <c r="C70" s="16" t="str">
         <f t="shared" si="7"/>
@@ -4220,7 +4706,7 @@
       </c>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A71" s="39"/>
+      <c r="A71" s="33"/>
       <c r="B71" s="12"/>
       <c r="C71" s="16" t="str">
         <f t="shared" si="7"/>
@@ -4258,7 +4744,7 @@
       </c>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A72" s="39"/>
+      <c r="A72" s="33"/>
       <c r="B72" s="12"/>
       <c r="C72" s="16" t="str">
         <f t="shared" si="7"/>
@@ -4296,7 +4782,7 @@
       </c>
     </row>
     <row r="73" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="39"/>
+      <c r="A73" s="33"/>
       <c r="B73" s="12"/>
       <c r="C73" s="16" t="str">
         <f t="shared" si="7"/>
@@ -4350,53 +4836,53 @@
       <c r="O74"/>
     </row>
     <row r="75" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A75" s="49" t="s">
+      <c r="A75" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="B75" s="49"/>
-      <c r="C75" s="49"/>
-      <c r="D75" s="49"/>
-      <c r="E75" s="49"/>
-      <c r="F75" s="49"/>
-      <c r="G75" s="49"/>
-      <c r="H75" s="49"/>
-      <c r="I75" s="49"/>
-      <c r="J75" s="49"/>
-      <c r="K75" s="49"/>
-      <c r="L75" s="49"/>
-      <c r="M75" s="49"/>
-      <c r="N75" s="49"/>
-      <c r="O75" s="49"/>
+      <c r="B75" s="41"/>
+      <c r="C75" s="41"/>
+      <c r="D75" s="41"/>
+      <c r="E75" s="41"/>
+      <c r="F75" s="41"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="41"/>
+      <c r="I75" s="41"/>
+      <c r="J75" s="41"/>
+      <c r="K75" s="41"/>
+      <c r="L75" s="41"/>
+      <c r="M75" s="41"/>
+      <c r="N75" s="41"/>
+      <c r="O75" s="41"/>
     </row>
     <row r="76" spans="1:15" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A76" s="1"/>
     </row>
     <row r="77" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
-      <c r="D77" s="45" t="s">
+      <c r="D77" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="E77" s="46"/>
-      <c r="F77" s="45" t="s">
+      <c r="E77" s="40"/>
+      <c r="F77" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="G77" s="46"/>
-      <c r="H77" s="45" t="s">
+      <c r="G77" s="40"/>
+      <c r="H77" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="I77" s="46"/>
-      <c r="J77" s="45" t="s">
+      <c r="I77" s="40"/>
+      <c r="J77" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="K77" s="46"/>
-      <c r="L77" s="45" t="s">
+      <c r="K77" s="40"/>
+      <c r="L77" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="M77" s="46"/>
-      <c r="N77" s="42" t="s">
+      <c r="M77" s="40"/>
+      <c r="N77" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="O77" s="43"/>
+      <c r="O77" s="37"/>
     </row>
     <row r="78" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B78" s="11" t="s">
@@ -4443,7 +4929,7 @@
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A79" s="39"/>
+      <c r="A79" s="33"/>
       <c r="B79" s="12"/>
       <c r="C79" s="16" t="str">
         <f>IF(ISBLANK($B79),"",SUM(D79,F79,H79,J79,L79,N79))</f>
@@ -4481,7 +4967,7 @@
       </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A80" s="39"/>
+      <c r="A80" s="33"/>
       <c r="B80" s="12"/>
       <c r="C80" s="16" t="str">
         <f t="shared" ref="C80:C109" si="14">IF(ISBLANK($B80),"",SUM(D80,F80,H80,J80,L80,N80))</f>
@@ -4519,7 +5005,7 @@
       </c>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A81" s="39"/>
+      <c r="A81" s="33"/>
       <c r="B81" s="12"/>
       <c r="C81" s="16" t="str">
         <f t="shared" si="14"/>
@@ -4557,7 +5043,7 @@
       </c>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A82" s="39"/>
+      <c r="A82" s="33"/>
       <c r="B82" s="12"/>
       <c r="C82" s="16" t="str">
         <f t="shared" si="14"/>
@@ -4595,7 +5081,7 @@
       </c>
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A83" s="39"/>
+      <c r="A83" s="33"/>
       <c r="B83" s="12"/>
       <c r="C83" s="16" t="str">
         <f t="shared" si="14"/>
@@ -4633,7 +5119,7 @@
       </c>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A84" s="39"/>
+      <c r="A84" s="33"/>
       <c r="B84" s="12"/>
       <c r="C84" s="16" t="str">
         <f t="shared" si="14"/>
@@ -4671,7 +5157,7 @@
       </c>
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A85" s="39"/>
+      <c r="A85" s="33"/>
       <c r="B85" s="12"/>
       <c r="C85" s="16" t="str">
         <f t="shared" si="14"/>
@@ -4709,7 +5195,7 @@
       </c>
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A86" s="39"/>
+      <c r="A86" s="33"/>
       <c r="B86" s="12"/>
       <c r="C86" s="16" t="str">
         <f t="shared" si="14"/>
@@ -4747,7 +5233,7 @@
       </c>
     </row>
     <row r="87" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A87" s="39"/>
+      <c r="A87" s="33"/>
       <c r="B87" s="12"/>
       <c r="C87" s="16" t="str">
         <f t="shared" si="14"/>
@@ -4785,143 +5271,311 @@
       </c>
     </row>
     <row r="88" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A88" s="39"/>
+      <c r="A88" s="33"/>
       <c r="B88" s="12"/>
-      <c r="C88" s="16"/>
+      <c r="C88" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
       <c r="D88" s="19"/>
-      <c r="E88" s="7"/>
+      <c r="E88" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
       <c r="F88" s="19"/>
-      <c r="G88" s="7"/>
+      <c r="G88" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
       <c r="H88" s="22"/>
-      <c r="I88" s="7"/>
+      <c r="I88" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
       <c r="J88" s="19"/>
-      <c r="K88" s="7"/>
+      <c r="K88" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
       <c r="L88" s="19"/>
-      <c r="M88" s="7"/>
+      <c r="M88" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
       <c r="N88" s="26"/>
-      <c r="O88" s="27"/>
+      <c r="O88" s="27" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
     </row>
     <row r="89" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A89" s="39"/>
+      <c r="A89" s="33"/>
       <c r="B89" s="12"/>
-      <c r="C89" s="16"/>
+      <c r="C89" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
       <c r="D89" s="19"/>
-      <c r="E89" s="7"/>
+      <c r="E89" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
       <c r="F89" s="19"/>
-      <c r="G89" s="7"/>
+      <c r="G89" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
       <c r="H89" s="22"/>
-      <c r="I89" s="7"/>
+      <c r="I89" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
       <c r="J89" s="19"/>
-      <c r="K89" s="7"/>
+      <c r="K89" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
       <c r="L89" s="19"/>
-      <c r="M89" s="7"/>
+      <c r="M89" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
       <c r="N89" s="26"/>
-      <c r="O89" s="27"/>
+      <c r="O89" s="27" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
     </row>
     <row r="90" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A90" s="39"/>
+      <c r="A90" s="33"/>
       <c r="B90" s="12"/>
-      <c r="C90" s="16"/>
+      <c r="C90" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
       <c r="D90" s="19"/>
-      <c r="E90" s="7"/>
+      <c r="E90" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
       <c r="F90" s="19"/>
-      <c r="G90" s="7"/>
+      <c r="G90" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
       <c r="H90" s="22"/>
-      <c r="I90" s="7"/>
+      <c r="I90" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
       <c r="J90" s="19"/>
-      <c r="K90" s="7"/>
+      <c r="K90" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
       <c r="L90" s="19"/>
-      <c r="M90" s="7"/>
+      <c r="M90" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
       <c r="N90" s="26"/>
-      <c r="O90" s="27"/>
+      <c r="O90" s="27" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
     </row>
     <row r="91" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A91" s="39"/>
+      <c r="A91" s="33"/>
       <c r="B91" s="12"/>
-      <c r="C91" s="16"/>
+      <c r="C91" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
       <c r="D91" s="19"/>
-      <c r="E91" s="7"/>
+      <c r="E91" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
       <c r="F91" s="19"/>
-      <c r="G91" s="7"/>
+      <c r="G91" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
       <c r="H91" s="22"/>
-      <c r="I91" s="7"/>
+      <c r="I91" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
       <c r="J91" s="19"/>
-      <c r="K91" s="7"/>
+      <c r="K91" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
       <c r="L91" s="19"/>
-      <c r="M91" s="7"/>
+      <c r="M91" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
       <c r="N91" s="26"/>
-      <c r="O91" s="27"/>
+      <c r="O91" s="27" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
     </row>
     <row r="92" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A92" s="39"/>
+      <c r="A92" s="33"/>
       <c r="B92" s="12"/>
-      <c r="C92" s="16"/>
+      <c r="C92" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
       <c r="D92" s="19"/>
-      <c r="E92" s="7"/>
+      <c r="E92" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
       <c r="F92" s="19"/>
-      <c r="G92" s="7"/>
+      <c r="G92" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
       <c r="H92" s="22"/>
-      <c r="I92" s="7"/>
+      <c r="I92" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
       <c r="J92" s="19"/>
-      <c r="K92" s="7"/>
+      <c r="K92" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
       <c r="L92" s="19"/>
-      <c r="M92" s="7"/>
+      <c r="M92" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
       <c r="N92" s="26"/>
-      <c r="O92" s="27"/>
+      <c r="O92" s="27" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
     </row>
     <row r="93" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A93" s="39"/>
+      <c r="A93" s="33"/>
       <c r="B93" s="12"/>
-      <c r="C93" s="16"/>
+      <c r="C93" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
       <c r="D93" s="19"/>
-      <c r="E93" s="7"/>
+      <c r="E93" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
       <c r="F93" s="19"/>
-      <c r="G93" s="7"/>
+      <c r="G93" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
       <c r="H93" s="22"/>
-      <c r="I93" s="7"/>
+      <c r="I93" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
       <c r="J93" s="19"/>
-      <c r="K93" s="7"/>
+      <c r="K93" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
       <c r="L93" s="19"/>
-      <c r="M93" s="7"/>
+      <c r="M93" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
       <c r="N93" s="26"/>
-      <c r="O93" s="27"/>
+      <c r="O93" s="27" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
     </row>
     <row r="94" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A94" s="39"/>
+      <c r="A94" s="33"/>
       <c r="B94" s="12"/>
-      <c r="C94" s="16"/>
+      <c r="C94" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
       <c r="D94" s="19"/>
-      <c r="E94" s="7"/>
+      <c r="E94" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
       <c r="F94" s="19"/>
-      <c r="G94" s="7"/>
+      <c r="G94" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
       <c r="H94" s="22"/>
-      <c r="I94" s="7"/>
+      <c r="I94" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
       <c r="J94" s="19"/>
-      <c r="K94" s="7"/>
+      <c r="K94" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
       <c r="L94" s="19"/>
-      <c r="M94" s="7"/>
+      <c r="M94" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
       <c r="N94" s="26"/>
-      <c r="O94" s="27"/>
+      <c r="O94" s="27" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
     </row>
     <row r="95" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A95" s="39"/>
+      <c r="A95" s="33"/>
       <c r="B95" s="12"/>
-      <c r="C95" s="16"/>
+      <c r="C95" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
       <c r="D95" s="19"/>
-      <c r="E95" s="7"/>
+      <c r="E95" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
       <c r="F95" s="19"/>
-      <c r="G95" s="7"/>
+      <c r="G95" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
       <c r="H95" s="22"/>
-      <c r="I95" s="7"/>
+      <c r="I95" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
       <c r="J95" s="19"/>
-      <c r="K95" s="7"/>
+      <c r="K95" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
       <c r="L95" s="19"/>
-      <c r="M95" s="7"/>
+      <c r="M95" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
       <c r="N95" s="26"/>
-      <c r="O95" s="27"/>
+      <c r="O95" s="27" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
     </row>
     <row r="96" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A96" s="39"/>
+      <c r="A96" s="33"/>
       <c r="B96" s="12"/>
       <c r="C96" s="16" t="str">
         <f t="shared" si="14"/>
@@ -4959,7 +5613,7 @@
       </c>
     </row>
     <row r="97" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A97" s="39"/>
+      <c r="A97" s="33"/>
       <c r="B97" s="12"/>
       <c r="C97" s="16" t="str">
         <f t="shared" si="14"/>
@@ -4997,7 +5651,7 @@
       </c>
     </row>
     <row r="98" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A98" s="39"/>
+      <c r="A98" s="33"/>
       <c r="B98" s="12"/>
       <c r="C98" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5035,7 +5689,7 @@
       </c>
     </row>
     <row r="99" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A99" s="39"/>
+      <c r="A99" s="33"/>
       <c r="B99" s="12"/>
       <c r="C99" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5073,7 +5727,7 @@
       </c>
     </row>
     <row r="100" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A100" s="39"/>
+      <c r="A100" s="33"/>
       <c r="B100" s="12"/>
       <c r="C100" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5111,7 +5765,7 @@
       </c>
     </row>
     <row r="101" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A101" s="39"/>
+      <c r="A101" s="33"/>
       <c r="B101" s="12"/>
       <c r="C101" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5149,7 +5803,7 @@
       </c>
     </row>
     <row r="102" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A102" s="39"/>
+      <c r="A102" s="33"/>
       <c r="B102" s="12"/>
       <c r="C102" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5187,7 +5841,7 @@
       </c>
     </row>
     <row r="103" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A103" s="39"/>
+      <c r="A103" s="33"/>
       <c r="B103" s="12"/>
       <c r="C103" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5225,7 +5879,7 @@
       </c>
     </row>
     <row r="104" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A104" s="39"/>
+      <c r="A104" s="33"/>
       <c r="B104" s="12"/>
       <c r="C104" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5263,7 +5917,7 @@
       </c>
     </row>
     <row r="105" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A105" s="39"/>
+      <c r="A105" s="33"/>
       <c r="B105" s="12"/>
       <c r="C105" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5301,7 +5955,7 @@
       </c>
     </row>
     <row r="106" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A106" s="39"/>
+      <c r="A106" s="33"/>
       <c r="B106" s="12"/>
       <c r="C106" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5339,7 +5993,7 @@
       </c>
     </row>
     <row r="107" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A107" s="39"/>
+      <c r="A107" s="33"/>
       <c r="B107" s="12"/>
       <c r="C107" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5377,7 +6031,7 @@
       </c>
     </row>
     <row r="108" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A108" s="39"/>
+      <c r="A108" s="33"/>
       <c r="B108" s="12"/>
       <c r="C108" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5415,7 +6069,7 @@
       </c>
     </row>
     <row r="109" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="39"/>
+      <c r="A109" s="33"/>
       <c r="B109" s="12"/>
       <c r="C109" s="16" t="str">
         <f t="shared" si="14"/>
@@ -5453,87 +6107,71 @@
       </c>
     </row>
     <row r="110" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B110" s="33"/>
-      <c r="C110" s="34"/>
-      <c r="D110" s="34"/>
-      <c r="E110" s="35"/>
-      <c r="F110" s="34"/>
-      <c r="G110" s="35"/>
-      <c r="H110" s="36"/>
-      <c r="I110" s="35"/>
-      <c r="J110" s="34"/>
-      <c r="K110" s="35"/>
-      <c r="L110" s="34"/>
-      <c r="M110" s="35"/>
-      <c r="N110" s="37"/>
-      <c r="O110" s="38"/>
+      <c r="A110" s="2"/>
+      <c r="B110" s="13"/>
+      <c r="C110" s="17"/>
+      <c r="D110" s="21"/>
+      <c r="E110" s="9"/>
+      <c r="F110" s="21"/>
+      <c r="G110" s="9"/>
+      <c r="H110" s="21"/>
     </row>
     <row r="111" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B111" s="33"/>
+      <c r="A111" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B111" s="34"/>
       <c r="C111" s="34"/>
       <c r="D111" s="34"/>
-      <c r="E111" s="35"/>
+      <c r="E111" s="34"/>
       <c r="F111" s="34"/>
-      <c r="G111" s="35"/>
-      <c r="H111" s="36"/>
-      <c r="I111" s="35"/>
+      <c r="G111" s="34"/>
+      <c r="H111" s="34"/>
+      <c r="I111" s="34"/>
       <c r="J111" s="34"/>
-      <c r="K111" s="35"/>
+      <c r="K111" s="34"/>
       <c r="L111" s="34"/>
-      <c r="M111" s="35"/>
-      <c r="N111" s="37"/>
-      <c r="O111" s="38"/>
-    </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A112" s="2"/>
-      <c r="B112" s="13"/>
-      <c r="C112" s="17"/>
-      <c r="D112" s="21"/>
-      <c r="E112" s="9"/>
-      <c r="F112" s="21"/>
-      <c r="G112" s="9"/>
-      <c r="H112" s="21"/>
+      <c r="M111" s="34"/>
+      <c r="N111" s="3"/>
+      <c r="O111" s="3"/>
     </row>
     <row r="113" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A113" s="40" t="s">
-        <v>0</v>
-      </c>
-      <c r="B113" s="40"/>
-      <c r="C113" s="40"/>
-      <c r="D113" s="40"/>
-      <c r="E113" s="40"/>
-      <c r="F113" s="40"/>
-      <c r="G113" s="40"/>
-      <c r="H113" s="40"/>
-      <c r="I113" s="40"/>
-      <c r="J113" s="40"/>
-      <c r="K113" s="40"/>
-      <c r="L113" s="40"/>
-      <c r="M113" s="40"/>
-      <c r="N113" s="3"/>
-      <c r="O113" s="3"/>
-    </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A115" s="41" t="s">
+      <c r="A113" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B115" s="41"/>
-      <c r="C115" s="41"/>
-      <c r="D115" s="41"/>
-      <c r="E115" s="41"/>
-      <c r="F115" s="41"/>
-      <c r="G115" s="41"/>
-      <c r="H115" s="41"/>
-      <c r="I115" s="41"/>
-      <c r="J115" s="41"/>
-      <c r="K115" s="41"/>
-      <c r="L115" s="41"/>
-      <c r="M115" s="41"/>
-      <c r="N115"/>
-      <c r="O115"/>
+      <c r="B113" s="35"/>
+      <c r="C113" s="35"/>
+      <c r="D113" s="35"/>
+      <c r="E113" s="35"/>
+      <c r="F113" s="35"/>
+      <c r="G113" s="35"/>
+      <c r="H113" s="35"/>
+      <c r="I113" s="35"/>
+      <c r="J113" s="35"/>
+      <c r="K113" s="35"/>
+      <c r="L113" s="35"/>
+      <c r="M113" s="35"/>
+      <c r="N113"/>
+      <c r="O113"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A113:M113"/>
+    <mergeCell ref="N5:O5"/>
+    <mergeCell ref="A3:O3"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="A7:A37"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="A111:M111"/>
+    <mergeCell ref="A39:O39"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="J41:K41"/>
+    <mergeCell ref="L41:M41"/>
     <mergeCell ref="A79:A109"/>
     <mergeCell ref="N41:O41"/>
     <mergeCell ref="A43:A73"/>
@@ -5544,22 +6182,6 @@
     <mergeCell ref="J77:K77"/>
     <mergeCell ref="L77:M77"/>
     <mergeCell ref="N77:O77"/>
-    <mergeCell ref="A115:M115"/>
-    <mergeCell ref="N5:O5"/>
-    <mergeCell ref="A3:O3"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="A7:A37"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="A113:M113"/>
-    <mergeCell ref="A39:O39"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="J41:K41"/>
-    <mergeCell ref="L41:M41"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5587,15 +6209,15 @@
       <c r="A2" s="1"/>
     </row>
     <row r="3" spans="1:7" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
     </row>
     <row r="4" spans="1:7" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
@@ -5617,7 +6239,7 @@
       <c r="G5"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="39"/>
+      <c r="A6" s="33"/>
       <c r="B6" s="12"/>
       <c r="C6" s="32" t="str">
         <f>IF(ISBLANK($B6),"",SUM(D6,E6,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5629,7 +6251,7 @@
       <c r="G6"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="39"/>
+      <c r="A7" s="33"/>
       <c r="B7" s="12"/>
       <c r="C7" s="32" t="str">
         <f>IF(ISBLANK($B7),"",SUM(D7,E7,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5641,7 +6263,7 @@
       <c r="G7"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="39"/>
+      <c r="A8" s="33"/>
       <c r="B8" s="12"/>
       <c r="C8" s="32" t="str">
         <f>IF(ISBLANK($B8),"",SUM(D8,E8,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5653,7 +6275,7 @@
       <c r="G8"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="39"/>
+      <c r="A9" s="33"/>
       <c r="B9" s="12"/>
       <c r="C9" s="32" t="str">
         <f>IF(ISBLANK($B9),"",SUM(D9,E9,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5665,7 +6287,7 @@
       <c r="G9"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="39"/>
+      <c r="A10" s="33"/>
       <c r="B10" s="12"/>
       <c r="C10" s="32" t="str">
         <f>IF(ISBLANK($B10),"",SUM(D10,E10,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5677,7 +6299,7 @@
       <c r="G10"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="39"/>
+      <c r="A11" s="33"/>
       <c r="B11" s="12"/>
       <c r="C11" s="32" t="str">
         <f>IF(ISBLANK($B11),"",SUM(D11,E11,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5689,7 +6311,7 @@
       <c r="G11"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="39"/>
+      <c r="A12" s="33"/>
       <c r="B12" s="12"/>
       <c r="C12" s="32" t="str">
         <f>IF(ISBLANK($B12),"",SUM(D12,E12,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5701,7 +6323,7 @@
       <c r="G12"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="39"/>
+      <c r="A13" s="33"/>
       <c r="B13" s="12"/>
       <c r="C13" s="32" t="str">
         <f>IF(ISBLANK($B13),"",SUM(D13,E13,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5713,7 +6335,7 @@
       <c r="G13"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="39"/>
+      <c r="A14" s="33"/>
       <c r="B14" s="12"/>
       <c r="C14" s="32" t="str">
         <f>IF(ISBLANK($B14),"",SUM(D14,E14,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5725,7 +6347,7 @@
       <c r="G14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="39"/>
+      <c r="A15" s="33"/>
       <c r="B15" s="12"/>
       <c r="C15" s="32" t="str">
         <f>IF(ISBLANK($B15),"",SUM(D15,E15,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5737,7 +6359,7 @@
       <c r="G15"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="39"/>
+      <c r="A16" s="33"/>
       <c r="B16" s="12"/>
       <c r="C16" s="32" t="str">
         <f>IF(ISBLANK($B16),"",SUM(D16,E16,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5749,88 +6371,115 @@
       <c r="G16"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="39"/>
+      <c r="A17" s="33"/>
       <c r="B17" s="12"/>
-      <c r="C17" s="32"/>
+      <c r="C17" s="32" t="str">
+        <f>IF(ISBLANK($B17),"",SUM(D17,E17,#REF!,#REF!,#REF!,#REF!))</f>
+        <v/>
+      </c>
       <c r="D17" s="32"/>
       <c r="E17" s="32"/>
       <c r="F17"/>
       <c r="G17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="39"/>
+      <c r="A18" s="33"/>
       <c r="B18" s="12"/>
-      <c r="C18" s="32"/>
+      <c r="C18" s="32" t="str">
+        <f>IF(ISBLANK($B18),"",SUM(D18,E18,#REF!,#REF!,#REF!,#REF!))</f>
+        <v/>
+      </c>
       <c r="D18" s="32"/>
       <c r="E18" s="32"/>
       <c r="F18"/>
       <c r="G18"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="39"/>
+      <c r="A19" s="33"/>
       <c r="B19" s="12"/>
-      <c r="C19" s="32"/>
+      <c r="C19" s="32" t="str">
+        <f>IF(ISBLANK($B19),"",SUM(D19,E19,#REF!,#REF!,#REF!,#REF!))</f>
+        <v/>
+      </c>
       <c r="D19" s="32"/>
       <c r="E19" s="32"/>
       <c r="F19"/>
       <c r="G19"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="39"/>
+      <c r="A20" s="33"/>
       <c r="B20" s="12"/>
-      <c r="C20" s="32"/>
+      <c r="C20" s="32" t="str">
+        <f>IF(ISBLANK($B20),"",SUM(D20,E20,#REF!,#REF!,#REF!,#REF!))</f>
+        <v/>
+      </c>
       <c r="D20" s="32"/>
       <c r="E20" s="32"/>
       <c r="F20"/>
       <c r="G20"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="39"/>
+      <c r="A21" s="33"/>
       <c r="B21" s="12"/>
-      <c r="C21" s="32"/>
+      <c r="C21" s="32" t="str">
+        <f>IF(ISBLANK($B21),"",SUM(D21,E21,#REF!,#REF!,#REF!,#REF!))</f>
+        <v/>
+      </c>
       <c r="D21" s="32"/>
       <c r="E21" s="32"/>
       <c r="F21"/>
       <c r="G21"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="39"/>
+      <c r="A22" s="33"/>
       <c r="B22" s="12"/>
-      <c r="C22" s="32"/>
+      <c r="C22" s="32" t="str">
+        <f>IF(ISBLANK($B22),"",SUM(D22,E22,#REF!,#REF!,#REF!,#REF!))</f>
+        <v/>
+      </c>
       <c r="D22" s="32"/>
       <c r="E22" s="32"/>
       <c r="F22"/>
       <c r="G22"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="39"/>
+      <c r="A23" s="33"/>
       <c r="B23" s="12"/>
-      <c r="C23" s="32"/>
+      <c r="C23" s="32" t="str">
+        <f>IF(ISBLANK($B23),"",SUM(D23,E23,#REF!,#REF!,#REF!,#REF!))</f>
+        <v/>
+      </c>
       <c r="D23" s="32"/>
       <c r="E23" s="32"/>
       <c r="F23"/>
       <c r="G23"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="39"/>
+      <c r="A24" s="33"/>
       <c r="B24" s="12"/>
-      <c r="C24" s="32"/>
+      <c r="C24" s="32" t="str">
+        <f>IF(ISBLANK($B24),"",SUM(D24,E24,#REF!,#REF!,#REF!,#REF!))</f>
+        <v/>
+      </c>
       <c r="D24" s="32"/>
       <c r="E24" s="32"/>
       <c r="F24"/>
       <c r="G24"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="39"/>
+      <c r="A25" s="33"/>
       <c r="B25" s="12"/>
-      <c r="C25" s="32"/>
+      <c r="C25" s="32" t="str">
+        <f>IF(ISBLANK($B25),"",SUM(D25,E25,#REF!,#REF!,#REF!,#REF!))</f>
+        <v/>
+      </c>
       <c r="D25" s="32"/>
       <c r="E25" s="32"/>
       <c r="F25"/>
       <c r="G25"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="39"/>
+      <c r="A26" s="33"/>
       <c r="B26" s="12"/>
       <c r="C26" s="32" t="str">
         <f>IF(ISBLANK($B26),"",SUM(D26,E26,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5842,7 +6491,7 @@
       <c r="G26"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="39"/>
+      <c r="A27" s="33"/>
       <c r="B27" s="12"/>
       <c r="C27" s="32" t="str">
         <f>IF(ISBLANK($B27),"",SUM(D27,E27,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5854,7 +6503,7 @@
       <c r="G27"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="39"/>
+      <c r="A28" s="33"/>
       <c r="B28" s="12"/>
       <c r="C28" s="32" t="str">
         <f>IF(ISBLANK($B28),"",SUM(D28,E28,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5866,7 +6515,7 @@
       <c r="G28"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="39"/>
+      <c r="A29" s="33"/>
       <c r="B29" s="12"/>
       <c r="C29" s="32" t="str">
         <f>IF(ISBLANK($B29),"",SUM(D29,E29,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5878,7 +6527,7 @@
       <c r="G29"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="39"/>
+      <c r="A30" s="33"/>
       <c r="B30" s="12"/>
       <c r="C30" s="32" t="str">
         <f>IF(ISBLANK($B30),"",SUM(D30,E30,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5890,7 +6539,7 @@
       <c r="G30"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="39"/>
+      <c r="A31" s="33"/>
       <c r="B31" s="12"/>
       <c r="C31" s="32" t="str">
         <f>IF(ISBLANK($B31),"",SUM(D31,E31,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5902,7 +6551,7 @@
       <c r="G31"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="39"/>
+      <c r="A32" s="33"/>
       <c r="B32" s="12"/>
       <c r="C32" s="32" t="str">
         <f>IF(ISBLANK($B32),"",SUM(D32,E32,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5914,7 +6563,7 @@
       <c r="G32"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="39"/>
+      <c r="A33" s="33"/>
       <c r="B33" s="12"/>
       <c r="C33" s="32" t="str">
         <f>IF(ISBLANK($B33),"",SUM(D33,E33,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5926,7 +6575,7 @@
       <c r="G33"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="39"/>
+      <c r="A34" s="33"/>
       <c r="B34" s="12"/>
       <c r="C34" s="32" t="str">
         <f>IF(ISBLANK($B34),"",SUM(D34,E34,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5938,7 +6587,7 @@
       <c r="G34"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="39"/>
+      <c r="A35" s="33"/>
       <c r="B35" s="12"/>
       <c r="C35" s="32" t="str">
         <f>IF(ISBLANK($B35),"",SUM(D35,E35,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5950,7 +6599,7 @@
       <c r="G35"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="39"/>
+      <c r="A36" s="33"/>
       <c r="B36" s="12"/>
       <c r="C36" s="32" t="str">
         <f>IF(ISBLANK($B36),"",SUM(D36,E36,#REF!,#REF!,#REF!,#REF!))</f>
@@ -5971,26 +6620,26 @@
       <c r="G37" s="21"/>
     </row>
     <row r="38" spans="1:7" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="40" t="s">
+      <c r="A38" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B38" s="40"/>
-      <c r="C38" s="40"/>
-      <c r="D38" s="40"/>
-      <c r="E38" s="40"/>
-      <c r="F38" s="40"/>
-      <c r="G38" s="40"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="34"/>
+      <c r="E38" s="34"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="34"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="41" t="s">
+      <c r="A40" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B40" s="41"/>
-      <c r="C40" s="41"/>
-      <c r="D40" s="41"/>
-      <c r="E40" s="41"/>
-      <c r="F40" s="41"/>
-      <c r="G40" s="41"/>
+      <c r="B40" s="35"/>
+      <c r="C40" s="35"/>
+      <c r="D40" s="35"/>
+      <c r="E40" s="35"/>
+      <c r="F40" s="35"/>
+      <c r="G40" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>